<commit_message>
Test PMS templates offline with synthetic data, signatures and logos
</commit_message>
<xml_diff>
--- a/examples/pms/invoice.xlsx
+++ b/examples/pms/invoice.xlsx
@@ -59,12 +59,12 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="914400" cy="609600"/>
+    <xdr:ext cx="1645920" cy="548640"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1" name="Picture 1" descr="{d.logo}"/>
@@ -79,7 +79,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="914400" cy="609600"/>
+          <a:ext cx="1645920" cy="548640"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -93,10 +93,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H13"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:D13"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
-    <col min="2" max="4" width="20" customWidth="1"/>
+    <col min="2" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="24" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -235,11 +239,14 @@
         </is>
       </c>
       <c r="D13">
-        <f>SUM(D11:D11)</f>
+        <f>SUM(D10:D12)</f>
         <v>0</v>
       </c>
     </row>
   </sheetData>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.2" footer="0.2"/>
+  <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
   <drawing r:id="rId70"/>
 </worksheet>
 </file>

</xml_diff>